<commit_message>
Update job ads chart labels
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-2_dataText/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jscott8\R Projects\lsip_dashboard\Data\3-2_dataText\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{50BC6191-9AF8-4D14-B309-FB400C7A4CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EF1EA43-A181-4023-B441-3C7796AC8001}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E79F000-3509-45F2-A178-B28243B787ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1820" yWindow="20" windowWidth="20660" windowHeight="14300" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
   <sheets>
     <sheet name="dataText" sheetId="1" r:id="rId1"/>
@@ -807,10 +807,10 @@
     <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. The total across geographies may not sum to the England total. The data includes minor instances of suppression in June and July 2025 due to quality concerns. Where this has occurred, only the data containing no suppression is included in the rolling average. ONS have partially imputed the data since October 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution. Additionally, a source of jobs was missing from the December 2025 and February 2026 data, and so some data has been suppressed in these months. Finally,  the entirety of the March 2026 data is currently supressed so is excluded from any three-month averages.</t>
   </si>
   <si>
-    <t>July 2026 data</t>
-  </si>
-  <si>
     <t>April 2025 - Mar 2026</t>
+  </si>
+  <si>
+    <t>August 2026 data</t>
   </si>
 </sst>
 </file>
@@ -1293,7 +1293,7 @@
         <v>152</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>22</v>
@@ -1334,7 +1334,7 @@
         <v>154</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>22</v>
@@ -1375,7 +1375,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>22</v>
@@ -1416,7 +1416,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>22</v>
@@ -1457,7 +1457,7 @@
         <v>153</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>22</v>
@@ -1498,7 +1498,7 @@
         <v>156</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>22</v>
@@ -1539,7 +1539,7 @@
         <v>157</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>22</v>
@@ -1580,7 +1580,7 @@
         <v>158</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>22</v>
@@ -1621,7 +1621,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>217</v>

</xml_diff>

<commit_message>
1) Changed metric name to "FE apprenticeship achievements" for clarity 2) Removed NA in the subheading 3) Changed name in datahub to "FE apprenticeship achievements volume"
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-2_dataText/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{6E79F000-3509-45F2-A178-B28243B787ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CC77C1D-A5E2-433B-B742-F316BB3F6D80}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{6E79F000-3509-45F2-A178-B28243B787ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55D7D6EA-0D99-4C14-BDFD-534B4183CB15}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="230">
   <si>
     <t>inactiveRate</t>
   </si>
@@ -941,7 +941,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -963,17 +963,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2239,41 +2228,43 @@
       <c r="G24" s="8"/>
     </row>
     <row r="25" spans="1:13" ht="232.5" thickBot="1">
-      <c r="A25" s="11" t="s">
+      <c r="A25" t="s">
         <v>220</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="11" t="s">
+      <c r="C25" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D25" t="s">
         <v>221</v>
       </c>
-      <c r="E25" s="12" t="s">
+      <c r="E25" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="G25" s="15" t="s">
+      <c r="G25" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="H25" s="15" t="s">
+      <c r="H25" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="I25" s="15" t="s">
+      <c r="I25" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="J25" s="15" t="s">
+      <c r="J25" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="K25" s="15" t="s">
+      <c r="K25" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="L25" s="15" t="s">
+      <c r="L25" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="M25" s="15" t="s">
+      <c r="M25" s="8" t="s">
         <v>227</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add further caveats to the top of the page. Uppercase SEND
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-2_dataText/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{1A40B41D-FC59-47BA-91C4-47EAE6F59AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA96CEFA-6828-48E1-A496-113F9AB70276}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{1A40B41D-FC59-47BA-91C4-47EAE6F59AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F004C54-FBEF-49B4-A84E-0EFE308D7650}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -875,10 +875,10 @@
     <t xml:space="preserve">This data is showing an estimate of the proportion of 16 and 17 year-olds  Not in Education or activity not known. Data is collected using the National Client Caseload Information System (NCCIS), which draws together local databases used to support young people to engage in education and training and plan services that meet young people’s needs. </t>
   </si>
   <si>
-    <t>NEET data is published at a Unitary Authority level, which is above the Local Authority District level shown in the maps and filters here. Therefore you will see missing data at the Local Authortity level in a number of places.</t>
-  </si>
-  <si>
     <t xml:space="preserve">These figures are estimates based on management information. Reported figures may be inaccurate due to local authority organisational changes or processing issues, resulting in missing or incorrect activity data for some young people. There is considerable variation at local authority level in how well 16 and 17 year olds are tracked, and hence ‘activity not known’ proportions can impact on the estimates of the proportion NEET. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEET/not known rates are shown here. Caution should be applied when using these figures due to the estimates being based on management information.  There is considerable variation in how well 16 and 17 year olds are tracked at local authority level. NEET data is published at a Unitary Authority level, which is above the Local Authority District level shown in the maps and filters here. Therefore you will see missing data at the Local Authortity level in a number of places. </t>
   </si>
 </sst>
 </file>
@@ -2306,7 +2306,7 @@
         <v>235</v>
       </c>
       <c r="C26" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D26" t="s">
         <v>236</v>
@@ -2315,7 +2315,7 @@
         <v>237</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>230</v>

</xml_diff>

<commit_message>
Update data notes for the NEET data after Harris QA.
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-2_dataText/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{1A40B41D-FC59-47BA-91C4-47EAE6F59AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE238A2E-0641-45C4-B453-F6906972D6AA}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{1A40B41D-FC59-47BA-91C4-47EAE6F59AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FAF2E69-65D9-4AD2-8C5A-5369CF5589EF}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -869,16 +869,19 @@
     <t>&lt;a href='https://explore-education-statistics.service.gov.uk/find-statistics/participation-in-education-training-and-neet-age-16-to-17-by-local-authority/2025-26'&gt;Participation in education, training and NEET age 16 to 17 by local authority&lt;/a&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">This data is showing an estimate of the proportion of 16 and 17 year-olds  Not in Education or activity not known. Data is collected using the National Client Caseload Information System (NCCIS), which draws together local databases used to support young people to engage in education and training and plan services that meet young people’s needs. </t>
-  </si>
-  <si>
     <t xml:space="preserve">These figures are estimates based on management information. Reported figures may be inaccurate due to local authority organisational changes or processing issues, resulting in missing or incorrect activity data for some young people. There is considerable variation at local authority level in how well 16 and 17 year olds are tracked, and hence ‘activity not known’ proportions can impact on the estimates of the proportion NEET. </t>
   </si>
   <si>
-    <t xml:space="preserve">NEET/not known rates are shown here. Caution should be applied when using these figures due to the estimates being based on management information.  There is considerable variation in how well 16 and 17 year olds are tracked at local authority level. NEET data is published at a Unitary Authority level, which is above the Local Authority District level shown in the maps and filters here. Therefore you will see missing data at the Local Authortity level in a number of places. </t>
-  </si>
-  <si>
     <t>Sept 2026 data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not in education or training (NEET)/not known rates are shown here. Caution should be applied when using these figures due to the estimates being based on management information.  There is considerable variation in how well 16 and 17 year olds are tracked at local authority level. NEET data is published at a Unitary Authority level, which is above the Local Authority District level shown in the maps and filters here. Therefore you will see missing data at the Local Authortity level in a number of places. </t>
+  </si>
+  <si>
+    <t>&lt;ol&gt;
+  &lt;li&gt;This data is showing an estimate of the proportion of 16 and 17 year-olds  NEET or activity not known. Data is collected using the National Client Caseload Information System (NCCIS), which draws together local databases used to support young people to engage in education and training and plan services that meet young people’s needs. &lt;/li&gt;
+&lt;li&gt; Although the source used is the best source for local level NEET data, there are other sources of NEET data. For example the &lt;a href='https://explore-education-statistics.service.gov.uk/find-statistics/neet-statistics-annual-brief/2025'&gt;national reporting that cover 16-24 year olds&lt;/a&gt;. &lt;/li&gt;
+&lt;/ol&gt;</t>
   </si>
 </sst>
 </file>
@@ -1689,7 +1692,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>211</v>
@@ -2298,7 +2301,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="160" thickBot="1">
+    <row r="26" spans="1:13" ht="305" thickBot="1">
       <c r="A26" t="s">
         <v>228</v>
       </c>
@@ -2312,10 +2315,10 @@
         <v>235</v>
       </c>
       <c r="E26" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>229</v>

</xml_diff>

<commit_message>
Make very minor text changes
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-2_dataText/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jscott8\R Projects\lsip_dashboard\Data\3-2_dataText\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{1A40B41D-FC59-47BA-91C4-47EAE6F59AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FAF2E69-65D9-4AD2-8C5A-5369CF5589EF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82889E7D-ABD8-4D1C-9844-F0B9922BF0E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
   <sheets>
     <sheet name="dataText" sheetId="1" r:id="rId1"/>
@@ -875,13 +875,13 @@
     <t>Sept 2026 data</t>
   </si>
   <si>
-    <t xml:space="preserve">Not in education or training (NEET)/not known rates are shown here. Caution should be applied when using these figures due to the estimates being based on management information.  There is considerable variation in how well 16 and 17 year olds are tracked at local authority level. NEET data is published at a Unitary Authority level, which is above the Local Authority District level shown in the maps and filters here. Therefore you will see missing data at the Local Authortity level in a number of places. </t>
-  </si>
-  <si>
     <t>&lt;ol&gt;
   &lt;li&gt;This data is showing an estimate of the proportion of 16 and 17 year-olds  NEET or activity not known. Data is collected using the National Client Caseload Information System (NCCIS), which draws together local databases used to support young people to engage in education and training and plan services that meet young people’s needs. &lt;/li&gt;
-&lt;li&gt; Although the source used is the best source for local level NEET data, there are other sources of NEET data. For example the &lt;a href='https://explore-education-statistics.service.gov.uk/find-statistics/neet-statistics-annual-brief/2025'&gt;national reporting that cover 16-24 year olds&lt;/a&gt;. &lt;/li&gt;
+&lt;li&gt; Although the source used is the best source for local level NEET data, there are other sources of NEET data. For example the &lt;a href='https://explore-education-statistics.service.gov.uk/find-statistics/neet-statistics-annual-brief/2025'&gt;national reporting that covers 16-24 year olds&lt;/a&gt;. &lt;/li&gt;
 &lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not in education or training (NEET)/not known rates are shown here. Caution should be applied when using these figures due to the estimates being based on management information. There is considerable variation in how well 16 and 17 year olds are tracked at local authority level. NEET data is published at a Unitary Authority level, which is above the Local Authority District level shown in the maps and filters here. Therefore you will see missing data at the Local Authortity level in a number of places. </t>
   </si>
 </sst>
 </file>
@@ -1311,11 +1311,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49D33D53-EEC7-4B18-8C67-5F9034426AB5}">
   <dimension ref="A1:M26"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="25" style="6" customWidth="1"/>
-    <col min="5" max="5" width="32.1796875" customWidth="1"/>
-    <col min="6" max="6" width="51.26953125" customWidth="1"/>
+    <col min="5" max="5" width="32.21875" customWidth="1"/>
+    <col min="6" max="6" width="51.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" thickBot="1">
@@ -1687,7 +1687,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="218" thickBot="1">
+    <row r="10" spans="1:13" ht="202.2" thickBot="1">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="145.5" thickBot="1">
+    <row r="11" spans="1:13" ht="130.19999999999999" thickBot="1">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="319.5" thickBot="1">
+    <row r="12" spans="1:13" ht="303" thickBot="1">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1810,7 +1810,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="319.5" thickBot="1">
+    <row r="13" spans="1:13" ht="303" thickBot="1">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="334" thickBot="1">
+    <row r="14" spans="1:13" ht="303" thickBot="1">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="319.5" thickBot="1">
+    <row r="15" spans="1:13" ht="303" thickBot="1">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="290.5" thickBot="1">
+    <row r="18" spans="1:13" ht="274.2" thickBot="1">
       <c r="A18" t="s">
         <v>160</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="290.5" thickBot="1">
+    <row r="19" spans="1:13" ht="259.8" thickBot="1">
       <c r="A19" t="s">
         <v>168</v>
       </c>
@@ -2097,7 +2097,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="263" thickBot="1">
+    <row r="20" spans="1:13" ht="289.8" thickBot="1">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -2138,7 +2138,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="254" thickBot="1">
+    <row r="21" spans="1:13" ht="280.2" thickBot="1">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="334" thickBot="1">
+    <row r="22" spans="1:13" ht="303" thickBot="1">
       <c r="A22" t="s">
         <v>159</v>
       </c>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="G23" s="8"/>
     </row>
-    <row r="24" spans="1:13" ht="363" thickBot="1">
+    <row r="24" spans="1:13" ht="331.8" thickBot="1">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="G24" s="8"/>
     </row>
-    <row r="25" spans="1:13" ht="232.5" thickBot="1">
+    <row r="25" spans="1:13" ht="216.6" thickBot="1">
       <c r="A25" t="s">
         <v>213</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="305" thickBot="1">
+    <row r="26" spans="1:13" ht="303" thickBot="1">
       <c r="A26" t="s">
         <v>228</v>
       </c>
@@ -2309,13 +2309,13 @@
         <v>234</v>
       </c>
       <c r="C26" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D26" t="s">
         <v>235</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>236</v>

</xml_diff>